<commit_message>
Added Qgen results to the test files
</commit_message>
<xml_diff>
--- a/src/tests/data/results/IEEE 30 bus.sav.xlsx
+++ b/src/tests/data/results/IEEE 30 bus.sav.xlsx
@@ -5,13 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
-    <sheet name="Vabs" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Vang" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="Pbranch" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="Qbranch" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="Vabs" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Vang" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Pbranch" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Qbranch" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Qgen" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="73">
   <si>
     <t xml:space="preserve">1</t>
   </si>
@@ -239,6 +240,9 @@
   </si>
   <si>
     <t xml:space="preserve">27_28_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MVAr</t>
   </si>
 </sst>
 </file>
@@ -329,13 +333,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -350,8 +358,114 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -367,7 +481,7 @@
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="2" t="n">
         <v>1.05999994277954</v>
       </c>
     </row>
@@ -375,7 +489,7 @@
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="2" t="n">
         <v>1.04499991168836</v>
       </c>
     </row>
@@ -383,7 +497,7 @@
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="2" t="n">
         <v>1.02117763781835</v>
       </c>
     </row>
@@ -391,7 +505,7 @@
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="2" t="n">
         <v>1.01230036792654</v>
       </c>
     </row>
@@ -399,7 +513,7 @@
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="2" t="n">
         <v>1.00999999249818</v>
       </c>
     </row>
@@ -407,7 +521,7 @@
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="2" t="n">
         <v>1.01062570429387</v>
       </c>
     </row>
@@ -415,7 +529,7 @@
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="2" t="n">
         <v>1.00259705029173</v>
       </c>
     </row>
@@ -423,7 +537,7 @@
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="2" t="n">
         <v>1.00999998129108</v>
       </c>
     </row>
@@ -431,7 +545,7 @@
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" s="2" t="n">
         <v>1.05113165464091</v>
       </c>
     </row>
@@ -439,7 +553,7 @@
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="2" t="n">
         <v>1.04537889818895</v>
       </c>
     </row>
@@ -447,7 +561,7 @@
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" s="2" t="n">
         <v>1.08199996535958</v>
       </c>
     </row>
@@ -455,7 +569,7 @@
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="0" t="n">
+      <c r="B13" s="2" t="n">
         <v>1.05733885405535</v>
       </c>
     </row>
@@ -463,7 +577,7 @@
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="0" t="n">
+      <c r="B14" s="2" t="n">
         <v>1.07100002040524</v>
       </c>
     </row>
@@ -471,7 +585,7 @@
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="0" t="n">
+      <c r="B15" s="2" t="n">
         <v>1.04250773898323</v>
       </c>
     </row>
@@ -479,7 +593,7 @@
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="0" t="n">
+      <c r="B16" s="2" t="n">
         <v>1.03791587573137</v>
       </c>
     </row>
@@ -487,7 +601,7 @@
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="0" t="n">
+      <c r="B17" s="2" t="n">
         <v>1.04462582784323</v>
       </c>
     </row>
@@ -495,7 +609,7 @@
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="0" t="n">
+      <c r="B18" s="2" t="n">
         <v>1.0401502793489</v>
       </c>
     </row>
@@ -503,7 +617,7 @@
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="0" t="n">
+      <c r="B19" s="2" t="n">
         <v>1.02839626742803</v>
       </c>
     </row>
@@ -511,7 +625,7 @@
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="0" t="n">
+      <c r="B20" s="2" t="n">
         <v>1.02589994495438</v>
       </c>
     </row>
@@ -519,7 +633,7 @@
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="0" t="n">
+      <c r="B21" s="2" t="n">
         <v>1.029986687839</v>
       </c>
     </row>
@@ -527,7 +641,7 @@
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="0" t="n">
+      <c r="B22" s="2" t="n">
         <v>1.03298218678066</v>
       </c>
     </row>
@@ -535,7 +649,7 @@
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="0" t="n">
+      <c r="B23" s="2" t="n">
         <v>1.03351363328317</v>
       </c>
     </row>
@@ -543,7 +657,7 @@
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="0" t="n">
+      <c r="B24" s="2" t="n">
         <v>1.02742897975398</v>
       </c>
     </row>
@@ -551,7 +665,7 @@
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="0" t="n">
+      <c r="B25" s="2" t="n">
         <v>1.02184577612474</v>
       </c>
     </row>
@@ -559,7 +673,7 @@
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="0" t="n">
+      <c r="B26" s="2" t="n">
         <v>1.01761861718844</v>
       </c>
     </row>
@@ -567,7 +681,7 @@
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="0" t="n">
+      <c r="B27" s="2" t="n">
         <v>0.999946367387374</v>
       </c>
     </row>
@@ -575,7 +689,7 @@
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="0" t="n">
+      <c r="B28" s="2" t="n">
         <v>1.0235384780157</v>
       </c>
     </row>
@@ -583,7 +697,7 @@
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="0" t="n">
+      <c r="B29" s="2" t="n">
         <v>1.00710102233856</v>
       </c>
     </row>
@@ -591,7 +705,7 @@
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="0" t="n">
+      <c r="B30" s="2" t="n">
         <v>1.0037057741359</v>
       </c>
     </row>
@@ -599,7 +713,7 @@
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="0" t="n">
+      <c r="B31" s="2" t="n">
         <v>0.992234779674377</v>
       </c>
     </row>
@@ -615,7 +729,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -631,7 +745,7 @@
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -639,7 +753,7 @@
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="2" t="n">
         <v>-0.0938680675279496</v>
       </c>
     </row>
@@ -647,7 +761,7 @@
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="2" t="n">
         <v>-0.131399914355754</v>
       </c>
     </row>
@@ -655,7 +769,7 @@
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="2" t="n">
         <v>-0.161956674411848</v>
       </c>
     </row>
@@ -663,7 +777,7 @@
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="2" t="n">
         <v>-0.246942610345029</v>
       </c>
     </row>
@@ -671,7 +785,7 @@
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="2" t="n">
         <v>-0.192946583491403</v>
       </c>
     </row>
@@ -679,7 +793,7 @@
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="2" t="n">
         <v>-0.224315306945025</v>
       </c>
     </row>
@@ -687,7 +801,7 @@
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="2" t="n">
         <v>-0.205903251917542</v>
       </c>
     </row>
@@ -695,7 +809,7 @@
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" s="2" t="n">
         <v>-0.246056021035836</v>
       </c>
     </row>
@@ -703,7 +817,7 @@
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="2" t="n">
         <v>-0.27381033443421</v>
       </c>
     </row>
@@ -711,7 +825,7 @@
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" s="2" t="n">
         <v>-0.246056014716265</v>
       </c>
     </row>
@@ -719,7 +833,7 @@
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="0" t="n">
+      <c r="B13" s="2" t="n">
         <v>-0.260628447856205</v>
       </c>
     </row>
@@ -727,7 +841,7 @@
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="0" t="n">
+      <c r="B14" s="2" t="n">
         <v>-0.260628441726585</v>
       </c>
     </row>
@@ -735,7 +849,7 @@
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="0" t="n">
+      <c r="B15" s="2" t="n">
         <v>-0.276190055976999</v>
       </c>
     </row>
@@ -743,7 +857,7 @@
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="0" t="n">
+      <c r="B16" s="2" t="n">
         <v>-0.277792981669785</v>
       </c>
     </row>
@@ -751,7 +865,7 @@
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="0" t="n">
+      <c r="B17" s="2" t="n">
         <v>-0.270795276358074</v>
       </c>
     </row>
@@ -759,7 +873,7 @@
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="0" t="n">
+      <c r="B18" s="2" t="n">
         <v>-0.276633809267762</v>
       </c>
     </row>
@@ -767,7 +881,7 @@
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="0" t="n">
+      <c r="B19" s="2" t="n">
         <v>-0.288506256058098</v>
       </c>
     </row>
@@ -775,7 +889,7 @@
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="0" t="n">
+      <c r="B20" s="2" t="n">
         <v>-0.291534982130216</v>
       </c>
     </row>
@@ -783,7 +897,7 @@
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="0" t="n">
+      <c r="B21" s="2" t="n">
         <v>-0.288104899606405</v>
       </c>
     </row>
@@ -791,7 +905,7 @@
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="0" t="n">
+      <c r="B22" s="2" t="n">
         <v>-0.281533267004714</v>
       </c>
     </row>
@@ -799,7 +913,7 @@
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="0" t="n">
+      <c r="B23" s="2" t="n">
         <v>-0.281284928888078</v>
       </c>
     </row>
@@ -807,7 +921,7 @@
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="0" t="n">
+      <c r="B24" s="2" t="n">
         <v>-0.284604342956748</v>
       </c>
     </row>
@@ -815,7 +929,7 @@
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="0" t="n">
+      <c r="B25" s="2" t="n">
         <v>-0.287678926455809</v>
       </c>
     </row>
@@ -823,7 +937,7 @@
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="0" t="n">
+      <c r="B26" s="2" t="n">
         <v>-0.28020495305378</v>
       </c>
     </row>
@@ -831,7 +945,7 @@
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="0" t="n">
+      <c r="B27" s="2" t="n">
         <v>-0.287525237336158</v>
       </c>
     </row>
@@ -839,7 +953,7 @@
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="0" t="n">
+      <c r="B28" s="2" t="n">
         <v>-0.271051067338068</v>
       </c>
     </row>
@@ -847,7 +961,7 @@
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="0" t="n">
+      <c r="B29" s="2" t="n">
         <v>-0.203807299206197</v>
       </c>
     </row>
@@ -855,7 +969,7 @@
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="0" t="n">
+      <c r="B30" s="2" t="n">
         <v>-0.292505231621384</v>
       </c>
     </row>
@@ -863,7 +977,7 @@
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="0" t="n">
+      <c r="B31" s="2" t="n">
         <v>-0.307904281470447</v>
       </c>
     </row>
@@ -879,14 +993,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B42"/>
   <sheetFormatPr defaultColWidth="9.01171875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="25.98"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -895,330 +1009,330 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="2" t="n">
         <v>173.30714</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="2" t="n">
         <v>87.6498</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="2" t="n">
         <v>43.65269</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="2" t="n">
         <v>82.36132</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="2" t="n">
         <v>60.37998</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="2" t="n">
         <v>82.1419</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="2" t="n">
         <v>72.12732</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="2" t="n">
         <v>-14.78171</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" s="2" t="n">
         <v>38.13212</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="2" t="n">
         <v>29.56305</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" s="2" t="n">
         <v>18.6735</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="0" t="n">
+      <c r="B13" s="2" t="n">
         <v>-0.54496</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="0" t="n">
+      <c r="B14" s="2" t="n">
         <v>5.33167</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="0" t="n">
+      <c r="B15" s="2" t="n">
         <v>9.02535</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B16" s="0" t="n">
+      <c r="B16" s="2" t="n">
         <v>15.78559</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="0" t="n">
+      <c r="B17" s="2" t="n">
         <v>7.6183</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B18" s="0" t="n">
+      <c r="B18" s="2" t="n">
         <v>7.85752</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B19" s="0" t="n">
+      <c r="B19" s="2" t="n">
         <v>17.89177</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="0" t="n">
+      <c r="B20" s="2" t="n">
         <v>7.24394</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="0" t="n">
+      <c r="B21" s="2" t="n">
         <v>1.58319</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B22" s="0" t="n">
+      <c r="B22" s="2" t="n">
         <v>6.01683</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="0" t="n">
+      <c r="B23" s="2" t="n">
         <v>5.03533</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="0" t="n">
+      <c r="B24" s="2" t="n">
         <v>3.6901</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B25" s="0" t="n">
+      <c r="B25" s="2" t="n">
         <v>2.77823</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="A26" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B26" s="0" t="n">
+      <c r="B26" s="2" t="n">
         <v>-6.72666</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B27" s="0" t="n">
+      <c r="B27" s="2" t="n">
         <v>-1.82568</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B28" s="0" t="n">
+      <c r="B28" s="2" t="n">
         <v>5.73935</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+      <c r="A29" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B29" s="0" t="n">
+      <c r="B29" s="2" t="n">
         <v>1.80394</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+      <c r="A30" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="0" t="n">
+      <c r="B30" s="2" t="n">
         <v>-1.20827</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B31" s="0" t="n">
+      <c r="B31" s="2" t="n">
         <v>3.54463</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+      <c r="A32" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B32" s="0" t="n">
+      <c r="B32" s="2" t="n">
         <v>-4.76285</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
+      <c r="A33" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B33" s="0" t="n">
+      <c r="B33" s="2" t="n">
         <v>6.18995</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
+      <c r="A34" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B34" s="0" t="n">
+      <c r="B34" s="2" t="n">
         <v>7.092</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+      <c r="A35" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B35" s="0" t="n">
+      <c r="B35" s="2" t="n">
         <v>3.70371</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
+      <c r="A36" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B36" s="0" t="n">
+      <c r="B36" s="2" t="n">
         <v>44.19323</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
+      <c r="A37" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B37" s="0" t="n">
+      <c r="B37" s="2" t="n">
         <v>27.72124</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
+      <c r="A38" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B38" s="0" t="n">
+      <c r="B38" s="2" t="n">
         <v>15.83966</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
+      <c r="A39" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B39" s="0" t="n">
+      <c r="B39" s="2" t="n">
         <v>18.06888</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="s">
+      <c r="A40" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B40" s="0" t="n">
+      <c r="B40" s="2" t="n">
         <v>27.72125</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
+      <c r="A41" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B41" s="0" t="n">
+      <c r="B41" s="2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="0" t="s">
+      <c r="A42" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B42" s="0" t="n">
+      <c r="B42" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1234,7 +1348,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -1250,7 +1364,7 @@
       <c r="A2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="2" t="n">
         <v>-24.7027912139893</v>
       </c>
     </row>
@@ -1258,7 +1372,7 @@
       <c r="A3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="2" t="n">
         <v>4.28486967086792</v>
       </c>
     </row>
@@ -1266,7 +1380,7 @@
       <c r="A4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="2" t="n">
         <v>4.74956703186035</v>
       </c>
     </row>
@@ -1274,7 +1388,7 @@
       <c r="A5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="2" t="n">
         <v>2.78163409233093</v>
       </c>
     </row>
@@ -1282,7 +1396,7 @@
       <c r="A6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="2" t="n">
         <v>1.37238574028015</v>
       </c>
     </row>
@@ -1290,7 +1404,7 @@
       <c r="A7" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="2" t="n">
         <v>-3.85462784767151</v>
       </c>
     </row>
@@ -1298,7 +1412,7 @@
       <c r="A8" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="2" t="n">
         <v>-15.9120197296143</v>
       </c>
     </row>
@@ -1306,7 +1420,7 @@
       <c r="A9" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="2" t="n">
         <v>11.4903240203857</v>
       </c>
     </row>
@@ -1314,7 +1428,7 @@
       <c r="A10" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" s="2" t="n">
         <v>-2.78136515617371</v>
       </c>
     </row>
@@ -1322,7 +1436,7 @@
       <c r="A11" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="2" t="n">
         <v>-7.19653463363647</v>
       </c>
     </row>
@@ -1330,7 +1444,7 @@
       <c r="A12" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" s="2" t="n">
         <v>0.114676266908646</v>
       </c>
     </row>
@@ -1338,7 +1452,7 @@
       <c r="A13" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="0" t="n">
+      <c r="B13" s="2" t="n">
         <v>-0.544621825218201</v>
       </c>
     </row>
@@ -1346,7 +1460,7 @@
       <c r="A14" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B14" s="0" t="n">
+      <c r="B14" s="2" t="n">
         <v>5.88191223144531</v>
       </c>
     </row>
@@ -1354,7 +1468,7 @@
       <c r="A15" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B15" s="0" t="n">
+      <c r="B15" s="2" t="n">
         <v>-15.5993537902832</v>
       </c>
     </row>
@@ -1362,7 +1476,7 @@
       <c r="A16" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="0" t="n">
+      <c r="B16" s="2" t="n">
         <v>4.42940664291382</v>
       </c>
     </row>
@@ -1370,7 +1484,7 @@
       <c r="A17" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B17" s="0" t="n">
+      <c r="B17" s="2" t="n">
         <v>3.70956254005432</v>
       </c>
     </row>
@@ -1378,7 +1492,7 @@
       <c r="A18" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="0" t="n">
+      <c r="B18" s="2" t="n">
         <v>10.0108547210693</v>
       </c>
     </row>
@@ -1386,7 +1500,7 @@
       <c r="A19" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B19" s="0" t="n">
+      <c r="B19" s="2" t="n">
         <v>4.60002613067627</v>
       </c>
     </row>
@@ -1394,7 +1508,7 @@
       <c r="A20" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B20" s="0" t="n">
+      <c r="B20" s="2" t="n">
         <v>-10.3174180984497</v>
       </c>
     </row>
@@ -1402,7 +1516,7 @@
       <c r="A21" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B21" s="0" t="n">
+      <c r="B21" s="2" t="n">
         <v>2.40030479431152</v>
       </c>
     </row>
@@ -1410,7 +1524,7 @@
       <c r="A22" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="0" t="n">
+      <c r="B22" s="2" t="n">
         <v>6.7899169921875</v>
       </c>
     </row>
@@ -1418,7 +1532,7 @@
       <c r="A23" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B23" s="0" t="n">
+      <c r="B23" s="2" t="n">
         <v>3.3485643863678</v>
       </c>
     </row>
@@ -1426,7 +1540,7 @@
       <c r="A24" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B24" s="0" t="n">
+      <c r="B24" s="2" t="n">
         <v>0.645794153213501</v>
       </c>
     </row>
@@ -1434,7 +1548,7 @@
       <c r="A25" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B25" s="0" t="n">
+      <c r="B25" s="2" t="n">
         <v>1.59529912471771</v>
       </c>
     </row>
@@ -1442,7 +1556,7 @@
       <c r="A26" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B26" s="0" t="n">
+      <c r="B26" s="2" t="n">
         <v>2.90788221359253</v>
       </c>
     </row>
@@ -1450,7 +1564,7 @@
       <c r="A27" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="0" t="n">
+      <c r="B27" s="2" t="n">
         <v>1.43537056446075</v>
       </c>
     </row>
@@ -1458,7 +1572,7 @@
       <c r="A28" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B28" s="0" t="n">
+      <c r="B28" s="2" t="n">
         <v>0.616709232330322</v>
       </c>
     </row>
@@ -1466,7 +1580,7 @@
       <c r="A29" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B29" s="0" t="n">
+      <c r="B29" s="2" t="n">
         <v>-2.79318451881409</v>
       </c>
     </row>
@@ -1474,7 +1588,7 @@
       <c r="A30" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B30" s="0" t="n">
+      <c r="B30" s="2" t="n">
         <v>-1.42861878871918</v>
       </c>
     </row>
@@ -1482,7 +1596,7 @@
       <c r="A31" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="0" t="n">
+      <c r="B31" s="2" t="n">
         <v>3.06158328056335</v>
       </c>
     </row>
@@ -1490,7 +1604,7 @@
       <c r="A32" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B32" s="0" t="n">
+      <c r="B32" s="2" t="n">
         <v>1.24448418617248</v>
       </c>
     </row>
@@ -1498,7 +1612,7 @@
       <c r="A33" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B33" s="0" t="n">
+      <c r="B33" s="2" t="n">
         <v>2.01279997825623</v>
       </c>
     </row>
@@ -1506,7 +1620,7 @@
       <c r="A34" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B34" s="0" t="n">
+      <c r="B34" s="2" t="n">
         <v>2.36665916442871</v>
       </c>
     </row>
@@ -1514,7 +1628,7 @@
       <c r="A35" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B35" s="0" t="n">
+      <c r="B35" s="2" t="n">
         <v>-0.371234387159347</v>
       </c>
     </row>
@@ -1522,7 +1636,7 @@
       <c r="A36" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B36" s="0" t="n">
+      <c r="B36" s="2" t="n">
         <v>1.66878843307495</v>
       </c>
     </row>
@@ -1530,7 +1644,7 @@
       <c r="A37" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B37" s="0" t="n">
+      <c r="B37" s="2" t="n">
         <v>1.66277551651001</v>
       </c>
     </row>
@@ -1538,7 +1652,7 @@
       <c r="A38" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B38" s="0" t="n">
+      <c r="B38" s="2" t="n">
         <v>0.605859696865082</v>
       </c>
     </row>
@@ -1546,7 +1660,7 @@
       <c r="A39" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B39" s="0" t="n">
+      <c r="B39" s="2" t="n">
         <v>14.4100160598755</v>
       </c>
     </row>
@@ -1554,7 +1668,7 @@
       <c r="A40" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B40" s="0" t="n">
+      <c r="B40" s="2" t="n">
         <v>-8.09298419952393</v>
       </c>
     </row>
@@ -1562,7 +1676,7 @@
       <c r="A41" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B41" s="0" t="n">
+      <c r="B41" s="2" t="n">
         <v>0.186543717980385</v>
       </c>
     </row>
@@ -1570,7 +1684,7 @@
       <c r="A42" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B42" s="0" t="n">
+      <c r="B42" s="2" t="n">
         <v>-3.74879360198975</v>
       </c>
     </row>
@@ -1583,4 +1697,76 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="0" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>-20.4176</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>56.0691</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>35.6585</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>36.111</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>16.0574</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>10.4507</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>